<commit_message>
Expand simulated demo network
</commit_message>
<xml_diff>
--- a/data/simulated/simulated_customer_network.xlsx
+++ b/data/simulated/simulated_customer_network.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,6 +429,27 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>CUST_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CUST_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CUST_8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CUST_10</t>
         </is>
       </c>
     </row>
@@ -443,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +626,299 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>2025-03-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CUST_6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CUST_6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EID_2222</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CUST_7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CUST_7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EID_2222</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CUST_8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CUST_8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-03-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CUST_10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CUST_10</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EID_5555</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CUST_11</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CUST_11</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EID_5555</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025-04-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CUST_12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CUST_12</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EID_5555</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2025-04-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CUST_13</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CUST_13</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EID_1313</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CUST_14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CUST_14</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EID_1414</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-04-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CUST_15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CUST_15</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EID_1515</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CUST_16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CUST_16</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EID_1616</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-04-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CUST_17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CUST_17</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EID_1717</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-04-18</t>
         </is>
       </c>
     </row>
@@ -619,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -834,6 +1148,306 @@
         <v>400</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CUST_11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TXN_101</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-02-01 10:00:00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HUB_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INBOUND</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CUST_13</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TXN_102</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:00:00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>HUB_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CUST_14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TXN_103</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HUB_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CUST_13</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TXN_104</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-02-04 13:00:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>JKL_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>INBOUND</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CUST_15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TXN_105</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-02-05 14:00:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>JKL_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CUST_14</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TXN_106</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-02-06 15:00:00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MNO_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INBOUND</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CUST_16</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TXN_107</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-02-07 16:00:00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MNO_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CUST_12</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TXN_108</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-02-08 17:00:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PQR_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>INBOUND</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CUST_17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TXN_109</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-02-09 18:00:00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PQR_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CUST_6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TXN_201</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-03-01 10:00:00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SOLO_ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>